<commit_message>
diário de bordo, atualização de currículo e criação de site para apresentação
</commit_message>
<xml_diff>
--- a/2024-08-01/Pixel art excel.xlsx
+++ b/2024-08-01/Pixel art excel.xlsx
@@ -25,7 +25,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -36,6 +36,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -269,7 +277,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -324,6 +332,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -611,6 +620,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:V181"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="10" max="13" width="9.140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="3:21" x14ac:dyDescent="0.25">
       <c r="C1" s="1"/>
@@ -1467,7 +1479,7 @@
       <c r="N41" s="22"/>
       <c r="O41" s="37"/>
       <c r="P41" s="25"/>
-      <c r="Q41" s="25"/>
+      <c r="Q41" s="54"/>
       <c r="R41" s="5"/>
       <c r="S41" s="5"/>
       <c r="T41" s="5"/>
@@ -1671,9 +1683,9 @@
       <c r="H51" s="5"/>
       <c r="I51" s="22"/>
       <c r="J51" s="22"/>
-      <c r="K51" s="22"/>
+      <c r="K51" s="5"/>
       <c r="L51" s="5"/>
-      <c r="M51" s="22"/>
+      <c r="M51" s="5"/>
       <c r="N51" s="22"/>
       <c r="O51" s="7"/>
       <c r="P51" s="5"/>

</xml_diff>